<commit_message>
docs: 명세 v4 후속 - 코드대조 4건 보정 (No.51 retry_after / No.52 verify 응답 / No.57 알림설정 필드 / No.60 DELETE 204)
</commit_message>
<xml_diff>
--- a/docs/api/api-spec-final.xlsx
+++ b/docs/api/api-spec-final.xlsx
@@ -7365,13 +7365,13 @@
       <c r="P55" s="33" t="inlineStr">
         <is>
           <t>{
-  "detail": "인증 코드가 발송되었습니다."
+  "detail": "인증 코드가 이메일로 발송되었습니다."
 }</t>
         </is>
       </c>
       <c r="Q55" s="33" t="inlineStr">
         <is>
-          <t>200 OK / 400 이메일 형식 오류 / 429 발송 쿨다운</t>
+          <t>200 OK / 400 이메일 형식 오류 / 429 발송 쿨다운 (body: {detail, retry_after})</t>
         </is>
       </c>
       <c r="R55" s="33" t="inlineStr">
@@ -7466,7 +7466,7 @@
       <c r="P56" s="33" t="inlineStr">
         <is>
           <t>{
-  "verified": true
+  "detail": "이메일 인증이 완료되었습니다."
 }</t>
         </is>
       </c>
@@ -7964,10 +7964,10 @@
       <c r="P61" s="33" t="inlineStr">
         <is>
           <t>{
-  "medication_alarm": true,
-  "challenge_alarm": true,
   "guide_complete_alarm": true,
-  "push_permission": true
+  "ocr_complete_alarm": true,
+  "system_alarm": true,
+  "updated_at": "2026-06-04T10:00:00Z"
 }</t>
         </is>
       </c>
@@ -8269,14 +8269,12 @@
       <c r="O64" s="33" t="n"/>
       <c r="P64" s="33" t="inlineStr">
         <is>
-          <t>{
-  "detail": "삭제되었습니다."
-}</t>
+          <t>204 No Content (응답 본문 없음)</t>
         </is>
       </c>
       <c r="Q64" s="33" t="inlineStr">
         <is>
-          <t>200 OK / 401 인증 실패 / 403 권한 없음 / 404 기록 없음</t>
+          <t>204 No Content / 401 인증 실패 / 403 권한 없음 / 404 기록 없음</t>
         </is>
       </c>
       <c r="R64" s="33" t="inlineStr">

</xml_diff>

<commit_message>
fix: develop(#110) 최신 명세에 No.43 보정 재적용 (xlsx 충돌 해소)
</commit_message>
<xml_diff>
--- a/docs/api/api-spec-final.xlsx
+++ b/docs/api/api-spec-final.xlsx
@@ -3046,7 +3046,17 @@
   "record_id": 10,
   "record_type": "prescription",
   "status": "ocr_completed",
-  "ocr_confidence": 0.91
+  "file_url": "https://.../rx.png",
+  "file_name": "처방전.png",
+  "file_size": 123456,
+  "content_type": "image/png",
+  "ocr_text": "...",
+  "ocr_edited_text": null,
+  "ocr_confidence": 0.91,
+  "input_method": "upload",
+  "image_expires_at": "2026-09-01T00:00:00Z",
+  "uploaded_at": "2026-06-04T10:00:00Z",
+  "updated_at": "2026-06-04T10:05:00Z"
 }</t>
         </is>
       </c>
@@ -3777,12 +3787,12 @@
       </c>
       <c r="S20" s="33" t="inlineStr">
         <is>
-          <t>⭐ v4: 미구현 — ocr-result의 medication_candidates로 대체 추정 (확인 필요)</t>
+          <t>구현 완료 (Backend B). 응답 {record_id, medications:[{medication_id, drug_name, dosage, frequency, timing, duration, is_verified, ...}]}</t>
         </is>
       </c>
       <c r="T20" s="28" t="inlineStr">
         <is>
-          <t>미구현 (확인필요)</t>
+          <t>완료</t>
         </is>
       </c>
     </row>
@@ -4082,12 +4092,12 @@
       </c>
       <c r="S23" s="33" t="inlineStr">
         <is>
-          <t>⭐ v4: 미구현 — GET /guides/{guide_id}로 대체 (확인 필요)</t>
+          <t>구현 완료 (#104, Backend B). 응답은 GET /guides/{guide_id}와 동일 (GenerateGuideResponse)</t>
         </is>
       </c>
       <c r="T23" s="28" t="inlineStr">
         <is>
-          <t>미구현 (확인필요)</t>
+          <t>완료</t>
         </is>
       </c>
     </row>
@@ -7357,13 +7367,13 @@
       <c r="P55" s="33" t="inlineStr">
         <is>
           <t>{
-  "detail": "인증 코드가 발송되었습니다."
+  "detail": "인증 코드가 이메일로 발송되었습니다."
 }</t>
         </is>
       </c>
       <c r="Q55" s="33" t="inlineStr">
         <is>
-          <t>200 OK / 400 이메일 형식 오류 / 429 발송 쿨다운</t>
+          <t>200 OK / 400 이메일 형식 오류 / 429 발송 쿨다운 (body: {detail, retry_after})</t>
         </is>
       </c>
       <c r="R55" s="33" t="inlineStr">
@@ -7458,7 +7468,7 @@
       <c r="P56" s="33" t="inlineStr">
         <is>
           <t>{
-  "verified": true
+  "detail": "이메일 인증이 완료되었습니다."
 }</t>
         </is>
       </c>
@@ -7956,10 +7966,10 @@
       <c r="P61" s="33" t="inlineStr">
         <is>
           <t>{
-  "medication_alarm": true,
-  "challenge_alarm": true,
   "guide_complete_alarm": true,
-  "push_permission": true
+  "ocr_complete_alarm": true,
+  "system_alarm": true,
+  "updated_at": "2026-06-04T10:00:00Z"
 }</t>
         </is>
       </c>
@@ -8261,14 +8271,12 @@
       <c r="O64" s="33" t="n"/>
       <c r="P64" s="33" t="inlineStr">
         <is>
-          <t>{
-  "detail": "삭제되었습니다."
-}</t>
+          <t>204 No Content (응답 본문 없음)</t>
         </is>
       </c>
       <c r="Q64" s="33" t="inlineStr">
         <is>
-          <t>200 OK / 401 인증 실패 / 403 권한 없음 / 404 기록 없음</t>
+          <t>204 No Content / 401 인증 실패 / 403 권한 없음 / 404 기록 없음</t>
         </is>
       </c>
       <c r="R64" s="33" t="inlineStr">

</xml_diff>

<commit_message>
docs: 명세 No.43 PUT notification-settings Request/Response 실제 DTO 필드로 보정 (#113)
* docs: 명세 No.43 PUT notification-settings Request/Response 실제 DTO 필드로 보정

* fix: develop(#110) 최신 명세에 No.43 보정 재적용 (xlsx 충돌 해소)
</commit_message>
<xml_diff>
--- a/docs/api/api-spec-final.xlsx
+++ b/docs/api/api-spec-final.xlsx
@@ -6519,17 +6519,19 @@
       <c r="O47" s="18" t="inlineStr">
         <is>
           <t>{
-  "medication_alarm": true,
-  "challenge_alarm": true,
   "guide_complete_alarm": true,
-  "push_permission": true
+  "ocr_complete_alarm": true,
+  "system_alarm": true
 }</t>
         </is>
       </c>
       <c r="P47" s="18" t="inlineStr">
         <is>
           <t>{
-  "updated_at": "2026-05-08T17:00:00"
+  "guide_complete_alarm": true,
+  "ocr_complete_alarm": true,
+  "system_alarm": true,
+  "updated_at": "2026-06-04T13:00:00Z"
 }</t>
         </is>
       </c>

</xml_diff>